<commit_message>
Ajout des TRI inondation
</commit_message>
<xml_diff>
--- a/data/Centres_departements.xlsx
+++ b/data/Centres_departements.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://circlestrategy-my.sharepoint.com/personal/ilyes_arfa_circlestrategy_onmicrosoft_com/Documents/Bureau/CATMAP_Data_Marketing/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://circlestrategy-my.sharepoint.com/personal/ilyes_arfa_circlestrategy_onmicrosoft_com/Documents/Bureau/CATMAP_Data_Marketing/API/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{127BF5F6-75EB-4EA8-9570-BEEF6161806E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="23" documentId="8_{127BF5F6-75EB-4EA8-9570-BEEF6161806E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{562C9698-C53C-5152-B07E-CF3EBD06A42C}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{F51D74F7-B85B-47A9-9BB8-BE32AE7A69F2}"/>
   </bookViews>

</xml_diff>